<commit_message>
feat: agregar tableros y flujos de producción
</commit_message>
<xml_diff>
--- a/Sheet1.xlsx
+++ b/Sheet1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juan.cabello\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miguel.arroyo\Desktop\macros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D461EAC0-5C44-42A7-8F3C-A275A5712359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EC1830-FDB7-4C81-ABDF-F12E9F1DC689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4470" yWindow="4095" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
     <t>ID Cliente</t>
   </si>
@@ -98,81 +98,6 @@
   </si>
   <si>
     <t>626469-01</t>
-  </si>
-  <si>
-    <t>625022-01</t>
-  </si>
-  <si>
-    <t>627046-01</t>
-  </si>
-  <si>
-    <t>626472-01</t>
-  </si>
-  <si>
-    <t>626433-01</t>
-  </si>
-  <si>
-    <t>613366-01</t>
-  </si>
-  <si>
-    <t>626310-01</t>
-  </si>
-  <si>
-    <t>613556-01</t>
-  </si>
-  <si>
-    <t>82-104984-191</t>
-  </si>
-  <si>
-    <t>82-104984-122</t>
-  </si>
-  <si>
-    <t>82-110915-01</t>
-  </si>
-  <si>
-    <t>82-110915-06</t>
-  </si>
-  <si>
-    <t>82-110915-09</t>
-  </si>
-  <si>
-    <t>82-110915-11</t>
-  </si>
-  <si>
-    <t>82-110915-13</t>
-  </si>
-  <si>
-    <t>82-110915-16</t>
-  </si>
-  <si>
-    <t>626798-02</t>
-  </si>
-  <si>
-    <t>82-104984-124</t>
-  </si>
-  <si>
-    <t>82-104984-147</t>
-  </si>
-  <si>
-    <t>82-104984-189</t>
-  </si>
-  <si>
-    <t>82-104984-190</t>
-  </si>
-  <si>
-    <t>82-104984-142</t>
-  </si>
-  <si>
-    <t>48TM003414</t>
-  </si>
-  <si>
-    <t>82-104985-39</t>
-  </si>
-  <si>
-    <t>82-104985-41</t>
-  </si>
-  <si>
-    <t>MTY</t>
   </si>
 </sst>
 </file>
@@ -8177,655 +8102,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <f>VLOOKUP(E5,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D5" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="4">
-        <v>1200</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <f>VLOOKUP(E6,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D6" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="4">
-        <v>600</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <f>VLOOKUP(E7,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D7" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="4">
-        <v>600</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="2" t="str">
-        <f>VLOOKUP(E8,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D8" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="4">
-        <v>600</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="2" t="str">
-        <f>VLOOKUP(E9,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D9" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="4">
-        <v>600</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="2" t="str">
-        <f>VLOOKUP(E10,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D10" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="4">
-        <v>600</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="2" t="str">
-        <f>VLOOKUP(E11,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D11" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="4">
-        <v>600</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="2" t="str">
-        <f>VLOOKUP(E12,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D12" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="4">
-        <v>518</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2" t="str">
-        <f>VLOOKUP(E13,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D13" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F13" s="4">
-        <v>100</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="2" t="str">
-        <f>VLOOKUP(E14,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM CIP-3501</v>
-      </c>
-      <c r="D14" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="4">
-        <v>320</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="2" t="str">
-        <f>VLOOKUP(E15,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM CIP-3501</v>
-      </c>
-      <c r="D15" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="4">
-        <v>312</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="2" t="str">
-        <f>VLOOKUP(E16,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM CIP-3501</v>
-      </c>
-      <c r="D16" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F16" s="4">
-        <v>468</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="2" t="str">
-        <f>VLOOKUP(E17,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM CIP-3501</v>
-      </c>
-      <c r="D17" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F17" s="4">
-        <v>210</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="2" t="str">
-        <f>VLOOKUP(E18,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM CIP-3501</v>
-      </c>
-      <c r="D18" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F18" s="4">
-        <v>616</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="2" t="str">
-        <f>VLOOKUP(E19,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM CIP-3501</v>
-      </c>
-      <c r="D19" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" s="4">
-        <v>216</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="2" t="str">
-        <f>VLOOKUP(E20,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>LENNOX 1</v>
-      </c>
-      <c r="D20" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F20" s="4">
-        <v>288</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="2" t="str">
-        <f>VLOOKUP(E21,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D21" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="4">
-        <v>100</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="2" t="str">
-        <f>VLOOKUP(E22,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D22" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="4">
-        <v>350</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="2" t="str">
-        <f>VLOOKUP(E23,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D23" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F23" s="4">
-        <v>247</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="2" t="str">
-        <f>VLOOKUP(E24,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D24" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F24" s="4">
-        <v>247</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="2" t="str">
-        <f>VLOOKUP(E25,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D25" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="4">
-        <v>700</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="2" t="str">
-        <f>VLOOKUP(E26,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D26" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F26" s="4">
-        <v>1400</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="2" t="str">
-        <f>VLOOKUP(E27,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D27" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F27" s="4">
-        <v>1500</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="2" t="str">
-        <f>VLOOKUP(E28,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D28" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F28" s="4">
-        <v>1000</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="2" t="e">
-        <f>VLOOKUP(E29,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D29" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F29" s="4">
-        <v>800</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="2" t="str">
-        <f>VLOOKUP(E30,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D30" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F30" s="4">
-        <v>300</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="2" t="str">
-        <f>VLOOKUP(E31,'[1]Sheet1 (2)'!$D$3:$L$307,9,0)</f>
-        <v>RHEEM TRANSFERENCIA</v>
-      </c>
-      <c r="D31" s="4">
-        <v>46262</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F31" s="4">
-        <v>6400</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="G32" s="2"/>

</xml_diff>